<commit_message>
New table for corotation. New plot for thesis (RRvsMM).
</commit_message>
<xml_diff>
--- a/tables/Important/Presentation.xlsx
+++ b/tables/Important/Presentation.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,12 +446,37 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>P_OB</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>P_orbit</t>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>P_OB_err</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Porb,ecl</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Porb,ecl_err</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>vsini_model</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>vsin(i)</t>
         </is>
       </c>
     </row>
@@ -473,10 +498,25 @@
         <v>4.8</v>
       </c>
       <c r="E2" t="n">
-        <v>2.562350433239974</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>2.087113936</v>
+        <v>2.375997674458885</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.2613715221114</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2.08704106</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3e-08</v>
+      </c>
+      <c r="J2" t="n">
+        <v>220</v>
+      </c>
+      <c r="K2" t="n">
+        <v>204.8</v>
       </c>
     </row>
     <row r="3">
@@ -497,10 +537,25 @@
         <v>526.8</v>
       </c>
       <c r="E3" t="n">
-        <v>4.204313305117789</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>3.728382</v>
+        <v>4.324436542406868</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.702374347557962</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3.728414</v>
+      </c>
+      <c r="I3" t="n">
+        <v>7.6e-06</v>
+      </c>
+      <c r="J3" t="n">
+        <v>140</v>
+      </c>
+      <c r="K3" t="n">
+        <v>224.9</v>
       </c>
     </row>
     <row r="4">
@@ -519,11 +574,24 @@
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>8.472035125887951</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
+        <v>4.09481697751251</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.4112528437837</v>
+      </c>
+      <c r="H4" t="n">
         <v>3.411581</v>
       </c>
+      <c r="I4" t="n">
+        <v>7e-06</v>
+      </c>
+      <c r="J4" t="n">
+        <v>240</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -543,10 +611,25 @@
         <v>13.5</v>
       </c>
       <c r="E5" t="n">
-        <v>1.450075842393898</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>1.40839776</v>
+        <v>1.238141680813251</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.0829473440097237</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.408379</v>
+      </c>
+      <c r="I5" t="n">
+        <v>7e-07</v>
+      </c>
+      <c r="J5" t="n">
+        <v>260</v>
+      </c>
+      <c r="K5" t="n">
+        <v>257.9</v>
       </c>
     </row>
     <row r="6">
@@ -567,10 +650,25 @@
         <v>0.71</v>
       </c>
       <c r="E6" t="n">
-        <v>4.036511806967425</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>3.89220909</v>
+        <v>3.941535058568192</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.357988858236117</v>
+      </c>
+      <c r="H6" t="n">
+        <v>3.89192316</v>
+      </c>
+      <c r="I6" t="n">
+        <v>6.6e-08</v>
+      </c>
+      <c r="J6" t="n">
+        <v>170</v>
+      </c>
+      <c r="K6" t="n">
+        <v>178</v>
       </c>
     </row>
     <row r="7">
@@ -591,10 +689,25 @@
         <v>283.2</v>
       </c>
       <c r="E7" t="n">
-        <v>13.4766741742306</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>8.964368</v>
+        <v>9.343827427466547</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.701607298175553</v>
+      </c>
+      <c r="H7" t="n">
+        <v>8.964427000000001</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1.2e-05</v>
+      </c>
+      <c r="J7" t="n">
+        <v>150</v>
+      </c>
+      <c r="K7" t="n">
+        <v>130.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>